<commit_message>
Scale UNICEF under-5 population values from thousands to absolute counts
</commit_message>
<xml_diff>
--- a/GBD_Input_Data_Package.xlsx
+++ b/GBD_Input_Data_Package.xlsx
@@ -492,7 +492,9 @@
           <t>MENA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="n">
+        <v>3168.762333333334</v>
+      </c>
       <c r="D2" t="n">
         <v>2.7</v>
       </c>
@@ -526,7 +528,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="n">
+        <v>4146.171333333333</v>
+      </c>
       <c r="D3" t="n">
         <v>19</v>
       </c>
@@ -560,7 +564,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>1450.962</v>
+      </c>
       <c r="D4" t="n">
         <v>19.6</v>
       </c>
@@ -594,7 +600,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>2234.092333333333</v>
+      </c>
       <c r="D5" t="n">
         <v>16.9</v>
       </c>
@@ -628,7 +636,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="n">
+        <v>2928.733666666667</v>
+      </c>
       <c r="D6" t="n">
         <v>11</v>
       </c>
@@ -662,7 +672,9 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="n">
+        <v>26.08933333333333</v>
+      </c>
       <c r="D7" t="n">
         <v>2.2</v>
       </c>
@@ -696,7 +708,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="n">
+        <v>2364.610666666667</v>
+      </c>
       <c r="D8" t="n">
         <v>18.2</v>
       </c>
@@ -730,7 +744,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="n">
+        <v>76.09666666666666</v>
+      </c>
       <c r="D9" t="n">
         <v>9.1</v>
       </c>
@@ -764,7 +780,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="n">
+        <v>168.2873333333334</v>
+      </c>
       <c r="D10" t="n">
         <v>5.6</v>
       </c>
@@ -798,7 +816,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="n">
+        <v>220.823</v>
+      </c>
       <c r="D11" t="n">
         <v>5.4</v>
       </c>
@@ -832,7 +852,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="n">
+        <v>255.7053333333333</v>
+      </c>
       <c r="D12" t="n">
         <v>11.6</v>
       </c>
@@ -866,7 +888,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="n">
+        <v>2817.177666666666</v>
+      </c>
       <c r="D13" t="n">
         <v>12</v>
       </c>
@@ -900,7 +924,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="n">
+        <v>1463.047</v>
+      </c>
       <c r="D14" t="n">
         <v>15</v>
       </c>
@@ -934,7 +960,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="n">
+        <v>198.199</v>
+      </c>
       <c r="D15" t="n">
         <v>18.8</v>
       </c>
@@ -968,7 +996,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="n">
+        <v>515.2873333333333</v>
+      </c>
       <c r="D16" t="n">
         <v>10.9</v>
       </c>
@@ -1002,7 +1032,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="n">
+        <v>3058.755</v>
+      </c>
       <c r="D17" t="n">
         <v>22.6</v>
       </c>
@@ -1036,7 +1068,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="n">
+        <v>2772.114666666666</v>
+      </c>
       <c r="D18" t="n">
         <v>15</v>
       </c>
@@ -1070,7 +1104,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="n">
+        <v>533.2773333333333</v>
+      </c>
       <c r="D19" t="n">
         <v>22.4</v>
       </c>
@@ -1104,7 +1140,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="n">
+        <v>40.37333333333333</v>
+      </c>
       <c r="D20" t="n">
         <v>13</v>
       </c>
@@ -1138,7 +1176,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="n">
+        <v>3111.434</v>
+      </c>
       <c r="D21" t="n">
         <v>34.6</v>
       </c>
@@ -1172,7 +1212,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>22351.083</v>
+      </c>
       <c r="D22" t="n">
         <v>24.4</v>
       </c>
@@ -1206,7 +1248,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="n">
+        <v>20.43266666666667</v>
+      </c>
       <c r="D23" t="n">
         <v>5.4</v>
       </c>
@@ -1240,7 +1284,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="n">
+        <v>1634.425666666667</v>
+      </c>
       <c r="D24" t="n">
         <v>16.2</v>
       </c>
@@ -1274,7 +1320,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="n">
+        <v>5.899999999999999</v>
+      </c>
       <c r="D25" t="n">
         <v>3.8</v>
       </c>
@@ -1308,7 +1356,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>775.8233333333333</v>
+      </c>
       <c r="D26" t="n">
         <v>12</v>
       </c>
@@ -1342,7 +1392,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="n">
+        <v>894.8136666666666</v>
+      </c>
       <c r="D27" t="n">
         <v>15.2</v>
       </c>
@@ -1376,7 +1428,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="n">
+        <v>1537.99</v>
+      </c>
       <c r="D28" t="n">
         <v>9.6</v>
       </c>
@@ -1410,7 +1464,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="n">
+        <v>195.7726666666667</v>
+      </c>
       <c r="D29" t="n">
         <v>11.8</v>
       </c>
@@ -1444,7 +1500,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" t="n">
+        <v>1444.822666666667</v>
+      </c>
       <c r="D30" t="n">
         <v>28.3</v>
       </c>
@@ -1478,7 +1536,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="n">
+        <v>627.2710000000001</v>
+      </c>
       <c r="D31" t="n">
         <v>18.4</v>
       </c>
@@ -1512,7 +1572,9 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
+      <c r="C32" t="n">
+        <v>590.4553333333333</v>
+      </c>
       <c r="D32" t="n">
         <v>12.3</v>
       </c>
@@ -1546,7 +1608,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
+      <c r="C33" t="n">
+        <v>3062.560666666667</v>
+      </c>
       <c r="D33" t="n">
         <v>13.6</v>
       </c>
@@ -1580,7 +1644,9 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="n">
+        <v>12850.584</v>
+      </c>
       <c r="D34" t="n">
         <v>25</v>
       </c>
@@ -1614,7 +1680,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="n">
+        <v>307.4083333333334</v>
+      </c>
       <c r="D35" t="n">
         <v>39.4</v>
       </c>
@@ -1648,7 +1716,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" t="n">
+        <v>12711.02</v>
+      </c>
       <c r="D36" t="n">
         <v>21.2</v>
       </c>
@@ -1682,7 +1752,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="n">
+        <v>4691.130666666667</v>
+      </c>
       <c r="D37" t="n">
         <v>9.800000000000001</v>
       </c>
@@ -1716,7 +1788,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" t="n">
+        <v>177.5583333333333</v>
+      </c>
       <c r="D38" t="n">
         <v>12.5</v>
       </c>
@@ -1750,7 +1824,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="n">
+        <v>2053.208333333333</v>
+      </c>
       <c r="D39" t="n">
         <v>12.8</v>
       </c>
@@ -1784,7 +1860,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="n">
+        <v>3779.074</v>
+      </c>
       <c r="D40" t="n">
         <v>15.4</v>
       </c>
@@ -1818,7 +1896,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="n">
+        <v>272.9746666666667</v>
+      </c>
       <c r="D41" t="n">
         <v>13.2</v>
       </c>
@@ -1852,7 +1932,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
+      <c r="C42" t="n">
+        <v>1252.289</v>
+      </c>
       <c r="D42" t="n">
         <v>7.7</v>
       </c>
@@ -1886,7 +1968,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
+      <c r="C43" t="n">
+        <v>3925.183666666666</v>
+      </c>
       <c r="D43" t="n">
         <v>4.9</v>
       </c>
@@ -1920,7 +2004,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="n">
+        <v>94.76733333333334</v>
+      </c>
       <c r="D44" t="n">
         <v>5</v>
       </c>
@@ -1954,7 +2040,9 @@
           <t>SSA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
+      <c r="C45" t="n">
+        <v>5292.233333333334</v>
+      </c>
       <c r="D45" t="n">
         <v>9.699999999999999</v>
       </c>
@@ -1988,7 +2076,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
+      <c r="C46" t="n">
+        <v>7206.933</v>
+      </c>
       <c r="D46" t="n">
         <v>11.4</v>
       </c>
@@ -2022,7 +2112,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
+      <c r="C47" t="n">
+        <v>2101.115333333333</v>
+      </c>
       <c r="D47" t="n">
         <v>11.8</v>
       </c>
@@ -2056,7 +2148,9 @@
           <t>LAC - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
+      <c r="C48" t="n">
+        <v>3.601666666666667</v>
+      </c>
       <c r="D48" t="n">
         <v>3.025</v>
       </c>
@@ -2090,7 +2184,9 @@
           <t>LAC - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
+      <c r="C49" t="n">
+        <v>1833.753</v>
+      </c>
       <c r="D49" t="n">
         <v>2</v>
       </c>
@@ -2124,7 +2220,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
+      <c r="C50" t="n">
+        <v>14.545</v>
+      </c>
       <c r="D50" t="n">
         <v>5.998924731182796</v>
       </c>
@@ -2158,7 +2256,9 @@
           <t>LAC - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="n">
+        <v>10.52933333333333</v>
+      </c>
       <c r="D51" t="n">
         <v>3.5</v>
       </c>
@@ -2192,7 +2292,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
+      <c r="C52" t="n">
+        <v>23.82533333333333</v>
+      </c>
       <c r="D52" t="n">
         <v>4.6</v>
       </c>
@@ -2226,7 +2328,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" t="n">
+        <v>8907.232666666667</v>
+      </c>
       <c r="D53" t="n">
         <v>3.5</v>
       </c>
@@ -2260,7 +2364,9 @@
           <t>LAC - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
+      <c r="C54" t="n">
+        <v>653.2093333333333</v>
+      </c>
       <c r="D54" t="n">
         <v>0.5</v>
       </c>
@@ -2294,7 +2400,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" t="n">
+        <v>2368.474</v>
+      </c>
       <c r="D55" t="n">
         <v>3.7</v>
       </c>
@@ -2328,7 +2436,9 @@
           <t>LAC - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
+      <c r="C56" t="n">
+        <v>189.4713333333333</v>
+      </c>
       <c r="D56" t="n">
         <v>2.9</v>
       </c>
@@ -2362,7 +2472,9 @@
           <t>LAC - High Child Mortality</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="n">
+        <v>2.436666666666667</v>
+      </c>
       <c r="D57" t="n">
         <v>7.569767441860465</v>
       </c>
@@ -2396,7 +2508,9 @@
           <t>LAC - High Child Mortality</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
+      <c r="C58" t="n">
+        <v>669.2916666666666</v>
+      </c>
       <c r="D58" t="n">
         <v>3</v>
       </c>
@@ -2430,7 +2544,9 @@
           <t>LAC - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" t="n">
+        <v>330.63</v>
+      </c>
       <c r="D59" t="n">
         <v>5</v>
       </c>
@@ -2464,7 +2580,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" t="n">
+        <v>4.648666666666666</v>
+      </c>
       <c r="D60" t="n">
         <v>5.998924731182796</v>
       </c>
@@ -2498,7 +2616,9 @@
           <t>LAC - High Child Mortality</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="n">
+        <v>55.27733333333333</v>
+      </c>
       <c r="D61" t="n">
         <v>9.4</v>
       </c>
@@ -2532,7 +2652,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" t="n">
+        <v>758.558</v>
+      </c>
       <c r="D62" t="n">
         <v>7.1</v>
       </c>
@@ -2566,7 +2688,9 @@
           <t>LAC - High Child Mortality</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
+      <c r="C63" t="n">
+        <v>110.3343333333333</v>
+      </c>
       <c r="D63" t="n">
         <v>2.5</v>
       </c>
@@ -2600,7 +2724,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
+      <c r="C64" t="n">
+        <v>6872.950333333333</v>
+      </c>
       <c r="D64" t="n">
         <v>4.2</v>
       </c>
@@ -2634,7 +2760,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
+      <c r="C65" t="n">
+        <v>239.854</v>
+      </c>
       <c r="D65" t="n">
         <v>2.9</v>
       </c>
@@ -2668,7 +2796,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
+      <c r="C66" t="n">
+        <v>452.8426666666667</v>
+      </c>
       <c r="D66" t="n">
         <v>1.3</v>
       </c>
@@ -2702,7 +2832,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
+      <c r="C67" t="n">
+        <v>1.891333333333334</v>
+      </c>
       <c r="D67" t="n">
         <v>5.998924731182796</v>
       </c>
@@ -2736,7 +2868,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
+      <c r="C68" t="n">
+        <v>6.806666666666668</v>
+      </c>
       <c r="D68" t="n">
         <v>2.8</v>
       </c>
@@ -2770,7 +2904,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
+      <c r="C69" t="n">
+        <v>4.247333333333334</v>
+      </c>
       <c r="D69" t="n">
         <v>5.998924731182796</v>
       </c>
@@ -2804,7 +2940,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
+      <c r="C70" t="n">
+        <v>35.55366666666666</v>
+      </c>
       <c r="D70" t="n">
         <v>6.7</v>
       </c>
@@ -2838,7 +2976,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
+      <c r="C71" t="n">
+        <v>56.21533333333333</v>
+      </c>
       <c r="D71" t="n">
         <v>4.9</v>
       </c>
@@ -2872,7 +3012,9 @@
           <t>LAC - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
+      <c r="C72" t="n">
+        <v>116.942</v>
+      </c>
       <c r="D72" t="n">
         <v>1.8</v>
       </c>
@@ -2906,7 +3048,9 @@
           <t>LAC - High Child Mortality</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
+      <c r="C73" t="n">
+        <v>1415.762666666667</v>
+      </c>
       <c r="D73" t="n">
         <v>2.9</v>
       </c>
@@ -2940,7 +3084,9 @@
           <t>LAC - High Child Mortality</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
+      <c r="C74" t="n">
+        <v>833.9530000000001</v>
+      </c>
       <c r="D74" t="n">
         <v>3.4</v>
       </c>
@@ -2974,7 +3120,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
+      <c r="C75" t="n">
+        <v>935.8233333333333</v>
+      </c>
       <c r="D75" t="n">
         <v>4.9</v>
       </c>
@@ -3008,7 +3156,9 @@
           <t>LAC - High Child Mortality</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
+      <c r="C76" t="n">
+        <v>1252.520333333333</v>
+      </c>
       <c r="D76" t="n">
         <v>14.4</v>
       </c>
@@ -3042,7 +3192,9 @@
           <t>LAC - High Child Mortality</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
+      <c r="C77" t="n">
+        <v>823.7020000000001</v>
+      </c>
       <c r="D77" t="n">
         <v>10.7</v>
       </c>
@@ -3076,7 +3228,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
+      <c r="C78" t="n">
+        <v>438.1393333333333</v>
+      </c>
       <c r="D78" t="n">
         <v>4.6</v>
       </c>
@@ -3110,7 +3264,9 @@
           <t>LAC - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
+      <c r="C79" t="n">
+        <v>1794.578666666667</v>
+      </c>
       <c r="D79" t="n">
         <v>2.7</v>
       </c>
@@ -3144,7 +3300,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
+      <c r="C80" t="n">
+        <v>63.13399999999999</v>
+      </c>
       <c r="D80" t="n">
         <v>7.6</v>
       </c>
@@ -3178,7 +3336,9 @@
           <t>ECA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
+      <c r="C81" t="n">
+        <v>49.36833333333333</v>
+      </c>
       <c r="D81" t="n">
         <v>1.445454545454546</v>
       </c>
@@ -3212,7 +3372,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
+      <c r="C82" t="n">
+        <v>4134.183</v>
+      </c>
       <c r="D82" t="n">
         <v>4.3</v>
       </c>
@@ -3246,7 +3408,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
+      <c r="C83" t="n">
+        <v>775.5136666666667</v>
+      </c>
       <c r="D83" t="n">
         <v>2.5</v>
       </c>
@@ -3280,7 +3444,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
+      <c r="C84" t="n">
+        <v>177.3906666666667</v>
+      </c>
       <c r="D84" t="n">
         <v>2.8</v>
       </c>
@@ -3314,7 +3480,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
+      <c r="C85" t="n">
+        <v>301.2693333333333</v>
+      </c>
       <c r="D85" t="n">
         <v>5.1</v>
       </c>
@@ -3348,7 +3516,9 @@
           <t>MENA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
+      <c r="C86" t="n">
+        <v>429.4949999999999</v>
+      </c>
       <c r="D86" t="n">
         <v>4.3</v>
       </c>
@@ -3382,7 +3552,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
+      <c r="C87" t="n">
+        <v>285.2923333333333</v>
+      </c>
       <c r="D87" t="n">
         <v>11.2</v>
       </c>
@@ -3416,7 +3588,9 @@
           <t>MENA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
+      <c r="C88" t="n">
+        <v>103.0066666666667</v>
+      </c>
       <c r="D88" t="n">
         <v>2.3</v>
       </c>
@@ -3450,7 +3624,9 @@
           <t>MENA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
+      <c r="C89" t="n">
+        <v>1742.14</v>
+      </c>
       <c r="D89" t="n">
         <v>3.5</v>
       </c>
@@ -3484,7 +3660,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
+      <c r="C90" t="n">
+        <v>1515.247666666667</v>
+      </c>
       <c r="D90" t="n">
         <v>10.4</v>
       </c>
@@ -3518,7 +3696,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
+      <c r="C91" t="n">
+        <v>601.3126666666667</v>
+      </c>
       <c r="D91" t="n">
         <v>1.6</v>
       </c>
@@ -3552,7 +3732,9 @@
           <t>MENA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
+      <c r="C92" t="n">
+        <v>382.1156666666666</v>
+      </c>
       <c r="D92" t="n">
         <v>4.461538461538462</v>
       </c>
@@ -3586,7 +3768,9 @@
           <t>SA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
+      <c r="C93" t="n">
+        <v>4437.454</v>
+      </c>
       <c r="D93" t="n">
         <v>4.53</v>
       </c>
@@ -3620,7 +3804,9 @@
           <t>MENA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
+      <c r="C94" t="n">
+        <v>76.33733333333333</v>
+      </c>
       <c r="D94" t="n">
         <v>17.7</v>
       </c>
@@ -3654,7 +3840,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
+      <c r="C95" t="n">
+        <v>7854.294666666666</v>
+      </c>
       <c r="D95" t="n">
         <v>3.7</v>
       </c>
@@ -3688,7 +3876,9 @@
           <t>MENA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
+      <c r="C96" t="n">
+        <v>3706.876333333334</v>
+      </c>
       <c r="D96" t="n">
         <v>3.9</v>
       </c>
@@ -3722,7 +3912,9 @@
           <t>MENA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
+      <c r="C97" t="n">
+        <v>2119.721</v>
+      </c>
       <c r="D97" t="n">
         <v>3</v>
       </c>
@@ -3756,7 +3948,9 @@
           <t>SA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
+      <c r="C98" t="n">
+        <v>21192.942</v>
+      </c>
       <c r="D98" t="n">
         <v>23.1</v>
       </c>
@@ -3790,7 +3984,9 @@
           <t>SSA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
+      <c r="C99" t="n">
+        <v>2274.471</v>
+      </c>
       <c r="D99" t="n">
         <v>22.5</v>
       </c>
@@ -3824,7 +4020,9 @@
           <t>SSA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
+      <c r="C100" t="n">
+        <v>5097.207333333333</v>
+      </c>
       <c r="D100" t="n">
         <v>33</v>
       </c>
@@ -3858,7 +4056,9 @@
           <t>MENA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
+      <c r="C101" t="n">
+        <v>4196.186333333334</v>
+      </c>
       <c r="D101" t="n">
         <v>40.7</v>
       </c>
@@ -3892,7 +4092,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
+      <c r="C102" t="n">
+        <v>14899.11633333333</v>
+      </c>
       <c r="D102" t="n">
         <v>15.9</v>
       </c>
@@ -3926,7 +4128,9 @@
           <t>SA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
+      <c r="C103" t="n">
+        <v>1090.037</v>
+      </c>
       <c r="D103" t="n">
         <v>17.1</v>
       </c>
@@ -3960,7 +4164,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
+      <c r="C104" t="n">
+        <v>2068.218333333334</v>
+      </c>
       <c r="D104" t="n">
         <v>6.7</v>
       </c>
@@ -3994,7 +4200,9 @@
           <t>EAP - High Child Mortality</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
+      <c r="C105" t="n">
+        <v>104.622</v>
+      </c>
       <c r="D105" t="n">
         <v>31.9</v>
       </c>
@@ -4028,7 +4236,9 @@
           <t>SA - High Child Mortality</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
+      <c r="C106" t="n">
+        <v>11003.37966666667</v>
+      </c>
       <c r="D106" t="n">
         <v>21.7</v>
       </c>
@@ -4062,7 +4272,9 @@
           <t>SA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
+      <c r="C107" t="n">
+        <v>32.21933333333333</v>
+      </c>
       <c r="D107" t="n">
         <v>8.699999999999999</v>
       </c>
@@ -4096,7 +4308,9 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
+      <c r="C108" t="n">
+        <v>1140.835333333333</v>
+      </c>
       <c r="D108" t="n">
         <v>9.300000000000001</v>
       </c>
@@ -4130,7 +4344,9 @@
           <t>SA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
+      <c r="C109" t="n">
+        <v>76443.10400000001</v>
+      </c>
       <c r="D109" t="n">
         <v>31.5</v>
       </c>
@@ -4164,7 +4380,9 @@
           <t>SA - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
+      <c r="C110" t="n">
+        <v>20.428</v>
+      </c>
       <c r="D110" t="n">
         <v>14.8</v>
       </c>
@@ -4198,7 +4416,9 @@
           <t>EAP - High Child Mortality</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr"/>
+      <c r="C111" t="n">
+        <v>2954.6</v>
+      </c>
       <c r="D111" t="n">
         <v>19.5</v>
       </c>
@@ -4232,7 +4452,9 @@
           <t>SA - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
+      <c r="C112" t="n">
+        <v>1861.383333333333</v>
+      </c>
       <c r="D112" t="n">
         <v>18.3</v>
       </c>
@@ -4266,7 +4488,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr"/>
+      <c r="C113" t="n">
+        <v>1210.857666666667</v>
+      </c>
       <c r="D113" t="n">
         <v>16.3</v>
       </c>
@@ -4300,7 +4524,9 @@
           <t>EAP - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
+      <c r="C114" t="n">
+        <v>38694.96933333333</v>
+      </c>
       <c r="D114" t="n">
         <v>2.4</v>
       </c>
@@ -4334,7 +4560,9 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr"/>
+      <c r="C115" t="n">
+        <v>0.6573333333333333</v>
+      </c>
       <c r="D115" t="n">
         <v>14.48334201388889</v>
       </c>
@@ -4368,7 +4596,9 @@
           <t>EAP - High Child Mortality</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr"/>
+      <c r="C116" t="n">
+        <v>55.10400000000001</v>
+      </c>
       <c r="D116" t="n">
         <v>4.6</v>
       </c>
@@ -4402,7 +4632,9 @@
           <t>EAP - High Child Mortality</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
+      <c r="C117" t="n">
+        <v>10.854</v>
+      </c>
       <c r="D117" t="n">
         <v>6.9</v>
       </c>
@@ -4436,7 +4668,9 @@
           <t>EAP - High Child Mortality</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
+      <c r="C118" t="n">
+        <v>530.462</v>
+      </c>
       <c r="D118" t="n">
         <v>24.3</v>
       </c>
@@ -4470,7 +4704,9 @@
           <t>EAP - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
+      <c r="C119" t="n">
+        <v>1514.116666666667</v>
+      </c>
       <c r="D119" t="n">
         <v>15.3</v>
       </c>
@@ -4504,7 +4740,9 @@
           <t>EAP - High Child Mortality</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
+      <c r="C120" t="n">
+        <v>2.858333333333333</v>
+      </c>
       <c r="D120" t="n">
         <v>11.9</v>
       </c>
@@ -4538,7 +4776,9 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
+      <c r="C121" t="n">
+        <v>8.086666666666668</v>
+      </c>
       <c r="D121" t="n">
         <v>14.48334201388889</v>
       </c>
@@ -4572,7 +4812,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
+      <c r="C122" t="n">
+        <v>235.3286666666667</v>
+      </c>
       <c r="D122" t="n">
         <v>1.9</v>
       </c>
@@ -4606,7 +4848,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr"/>
+      <c r="C123" t="n">
+        <v>0.9923333333333333</v>
+      </c>
       <c r="D123" t="n">
         <v>3.8</v>
       </c>
@@ -4640,7 +4884,9 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
+      <c r="C124" t="n">
+        <v>0.082</v>
+      </c>
       <c r="D124" t="n">
         <v>14.48334201388889</v>
       </c>
@@ -4674,7 +4920,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
+      <c r="C125" t="n">
+        <v>0.656</v>
+      </c>
       <c r="D125" t="n">
         <v>17.684</v>
       </c>
@@ -4708,7 +4956,9 @@
           <t>EAP - High Child Mortality</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
+      <c r="C126" t="n">
+        <v>819.1286666666666</v>
+      </c>
       <c r="D126" t="n">
         <v>27.8</v>
       </c>
@@ -4742,7 +4992,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
+      <c r="C127" t="n">
+        <v>6401.461333333333</v>
+      </c>
       <c r="D127" t="n">
         <v>16.7</v>
       </c>
@@ -4776,7 +5028,9 @@
           <t>EAP - Low Child Mortality</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
+      <c r="C128" t="n">
+        <v>905.511</v>
+      </c>
       <c r="D128" t="n">
         <v>0.4</v>
       </c>
@@ -4810,7 +5064,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr"/>
+      <c r="C129" t="n">
+        <v>18.856</v>
+      </c>
       <c r="D129" t="n">
         <v>3.4</v>
       </c>
@@ -4844,7 +5100,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr"/>
+      <c r="C130" t="n">
+        <v>69.12133333333334</v>
+      </c>
       <c r="D130" t="n">
         <v>16.2</v>
       </c>
@@ -4878,7 +5136,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr"/>
+      <c r="C131" t="n">
+        <v>7.870333333333334</v>
+      </c>
       <c r="D131" t="n">
         <v>0.8</v>
       </c>
@@ -4912,7 +5172,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr"/>
+      <c r="C132" t="n">
+        <v>0.7313333333333333</v>
+      </c>
       <c r="D132" t="n">
         <v>2.9</v>
       </c>
@@ -4946,7 +5208,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
+      <c r="C133" t="n">
+        <v>29.333</v>
+      </c>
       <c r="D133" t="n">
         <v>11.7</v>
       </c>
@@ -4980,7 +5244,9 @@
           <t>EAP - Medium Child Mortality</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
+      <c r="C134" t="n">
+        <v>4785.569666666666</v>
+      </c>
       <c r="D134" t="n">
         <v>9.699999999999999</v>
       </c>

</xml_diff>

<commit_message>
Fix UNICEF Under-5 population scaling: convert string values to float before multiplying by 1000
</commit_message>
<xml_diff>
--- a/GBD_Input_Data_Package.xlsx
+++ b/GBD_Input_Data_Package.xlsx
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3168.762333333334</v>
+        <v>3168762.333333333</v>
       </c>
       <c r="D2" t="n">
         <v>2.7</v>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4146.171333333333</v>
+        <v>4146171.333333333</v>
       </c>
       <c r="D3" t="n">
         <v>19</v>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1450.962</v>
+        <v>1450962</v>
       </c>
       <c r="D4" t="n">
         <v>19.6</v>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2234.092333333333</v>
+        <v>2234092.333333333</v>
       </c>
       <c r="D5" t="n">
         <v>16.9</v>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2928.733666666667</v>
+        <v>2928733.666666667</v>
       </c>
       <c r="D6" t="n">
         <v>11</v>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>26.08933333333333</v>
+        <v>26089.33333333333</v>
       </c>
       <c r="D7" t="n">
         <v>2.2</v>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2364.610666666667</v>
+        <v>2364610.666666667</v>
       </c>
       <c r="D8" t="n">
         <v>18.2</v>
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>76.09666666666666</v>
+        <v>76096.66666666667</v>
       </c>
       <c r="D9" t="n">
         <v>9.1</v>
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>168.2873333333334</v>
+        <v>168287.3333333333</v>
       </c>
       <c r="D10" t="n">
         <v>5.6</v>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>220.823</v>
+        <v>220823</v>
       </c>
       <c r="D11" t="n">
         <v>5.4</v>
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>255.7053333333333</v>
+        <v>255705.3333333333</v>
       </c>
       <c r="D12" t="n">
         <v>11.6</v>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2817.177666666666</v>
+        <v>2817177.666666667</v>
       </c>
       <c r="D13" t="n">
         <v>12</v>
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1463.047</v>
+        <v>1463047</v>
       </c>
       <c r="D14" t="n">
         <v>15</v>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>198.199</v>
+        <v>198199</v>
       </c>
       <c r="D15" t="n">
         <v>18.8</v>
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>515.2873333333333</v>
+        <v>515287.3333333333</v>
       </c>
       <c r="D16" t="n">
         <v>10.9</v>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3058.755</v>
+        <v>3058755</v>
       </c>
       <c r="D17" t="n">
         <v>22.6</v>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2772.114666666666</v>
+        <v>2772114.666666667</v>
       </c>
       <c r="D18" t="n">
         <v>15</v>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>533.2773333333333</v>
+        <v>533277.3333333334</v>
       </c>
       <c r="D19" t="n">
         <v>22.4</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>40.37333333333333</v>
+        <v>40373.33333333334</v>
       </c>
       <c r="D20" t="n">
         <v>13</v>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3111.434</v>
+        <v>3111434</v>
       </c>
       <c r="D21" t="n">
         <v>34.6</v>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22351.083</v>
+        <v>22351083</v>
       </c>
       <c r="D22" t="n">
         <v>24.4</v>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>20.43266666666667</v>
+        <v>20432.66666666667</v>
       </c>
       <c r="D23" t="n">
         <v>5.4</v>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1634.425666666667</v>
+        <v>1634425.666666667</v>
       </c>
       <c r="D24" t="n">
         <v>16.2</v>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>5.899999999999999</v>
+        <v>5900</v>
       </c>
       <c r="D25" t="n">
         <v>3.8</v>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>775.8233333333333</v>
+        <v>775823.3333333334</v>
       </c>
       <c r="D26" t="n">
         <v>12</v>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>894.8136666666666</v>
+        <v>894813.6666666666</v>
       </c>
       <c r="D27" t="n">
         <v>15.2</v>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1537.99</v>
+        <v>1537990</v>
       </c>
       <c r="D28" t="n">
         <v>9.6</v>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>195.7726666666667</v>
+        <v>195772.6666666667</v>
       </c>
       <c r="D29" t="n">
         <v>11.8</v>
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1444.822666666667</v>
+        <v>1444822.666666667</v>
       </c>
       <c r="D30" t="n">
         <v>28.3</v>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>627.2710000000001</v>
+        <v>627271</v>
       </c>
       <c r="D31" t="n">
         <v>18.4</v>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>590.4553333333333</v>
+        <v>590455.3333333334</v>
       </c>
       <c r="D32" t="n">
         <v>12.3</v>
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3062.560666666667</v>
+        <v>3062560.666666667</v>
       </c>
       <c r="D33" t="n">
         <v>13.6</v>
@@ -1645,7 +1645,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>12850.584</v>
+        <v>12850584</v>
       </c>
       <c r="D34" t="n">
         <v>25</v>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>307.4083333333334</v>
+        <v>307408.3333333333</v>
       </c>
       <c r="D35" t="n">
         <v>39.4</v>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>12711.02</v>
+        <v>12711020</v>
       </c>
       <c r="D36" t="n">
         <v>21.2</v>
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4691.130666666667</v>
+        <v>4691130.666666667</v>
       </c>
       <c r="D37" t="n">
         <v>9.800000000000001</v>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>177.5583333333333</v>
+        <v>177558.3333333333</v>
       </c>
       <c r="D38" t="n">
         <v>12.5</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2053.208333333333</v>
+        <v>2053208.333333333</v>
       </c>
       <c r="D39" t="n">
         <v>12.8</v>
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3779.074</v>
+        <v>3779074</v>
       </c>
       <c r="D40" t="n">
         <v>15.4</v>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>272.9746666666667</v>
+        <v>272974.6666666667</v>
       </c>
       <c r="D41" t="n">
         <v>13.2</v>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1252.289</v>
+        <v>1252289</v>
       </c>
       <c r="D42" t="n">
         <v>7.7</v>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3925.183666666666</v>
+        <v>3925183.666666667</v>
       </c>
       <c r="D43" t="n">
         <v>4.9</v>
@@ -2005,7 +2005,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>94.76733333333334</v>
+        <v>94767.33333333333</v>
       </c>
       <c r="D44" t="n">
         <v>5</v>
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>5292.233333333334</v>
+        <v>5292233.333333333</v>
       </c>
       <c r="D45" t="n">
         <v>9.699999999999999</v>
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>7206.933</v>
+        <v>7206933</v>
       </c>
       <c r="D46" t="n">
         <v>11.4</v>
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2101.115333333333</v>
+        <v>2101115.333333333</v>
       </c>
       <c r="D47" t="n">
         <v>11.8</v>
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3.601666666666667</v>
+        <v>3601.666666666667</v>
       </c>
       <c r="D48" t="n">
         <v>3.025</v>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1833.753</v>
+        <v>1833753</v>
       </c>
       <c r="D49" t="n">
         <v>2</v>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>14.545</v>
+        <v>14545</v>
       </c>
       <c r="D50" t="n">
         <v>5.998924731182796</v>
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>10.52933333333333</v>
+        <v>10529.33333333333</v>
       </c>
       <c r="D51" t="n">
         <v>3.5</v>
@@ -2293,7 +2293,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>23.82533333333333</v>
+        <v>23825.33333333333</v>
       </c>
       <c r="D52" t="n">
         <v>4.6</v>
@@ -2329,7 +2329,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>8907.232666666667</v>
+        <v>8907232.666666666</v>
       </c>
       <c r="D53" t="n">
         <v>3.5</v>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>653.2093333333333</v>
+        <v>653209.3333333334</v>
       </c>
       <c r="D54" t="n">
         <v>0.5</v>
@@ -2401,7 +2401,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2368.474</v>
+        <v>2368474</v>
       </c>
       <c r="D55" t="n">
         <v>3.7</v>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>189.4713333333333</v>
+        <v>189471.3333333333</v>
       </c>
       <c r="D56" t="n">
         <v>2.9</v>
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2.436666666666667</v>
+        <v>2436.666666666667</v>
       </c>
       <c r="D57" t="n">
         <v>7.569767441860465</v>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>669.2916666666666</v>
+        <v>669291.6666666666</v>
       </c>
       <c r="D58" t="n">
         <v>3</v>
@@ -2545,7 +2545,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>330.63</v>
+        <v>330630</v>
       </c>
       <c r="D59" t="n">
         <v>5</v>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4.648666666666666</v>
+        <v>4648.666666666667</v>
       </c>
       <c r="D60" t="n">
         <v>5.998924731182796</v>
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>55.27733333333333</v>
+        <v>55277.33333333334</v>
       </c>
       <c r="D61" t="n">
         <v>9.4</v>
@@ -2653,7 +2653,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>758.558</v>
+        <v>758558</v>
       </c>
       <c r="D62" t="n">
         <v>7.1</v>
@@ -2689,7 +2689,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>110.3343333333333</v>
+        <v>110334.3333333333</v>
       </c>
       <c r="D63" t="n">
         <v>2.5</v>
@@ -2725,7 +2725,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>6872.950333333333</v>
+        <v>6872950.333333333</v>
       </c>
       <c r="D64" t="n">
         <v>4.2</v>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>239.854</v>
+        <v>239854</v>
       </c>
       <c r="D65" t="n">
         <v>2.9</v>
@@ -2797,7 +2797,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>452.8426666666667</v>
+        <v>452842.6666666667</v>
       </c>
       <c r="D66" t="n">
         <v>1.3</v>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1.891333333333334</v>
+        <v>1891.333333333333</v>
       </c>
       <c r="D67" t="n">
         <v>5.998924731182796</v>
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>6.806666666666668</v>
+        <v>6806.666666666667</v>
       </c>
       <c r="D68" t="n">
         <v>2.8</v>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>4.247333333333334</v>
+        <v>4247.333333333333</v>
       </c>
       <c r="D69" t="n">
         <v>5.998924731182796</v>
@@ -2941,7 +2941,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>35.55366666666666</v>
+        <v>35553.66666666666</v>
       </c>
       <c r="D70" t="n">
         <v>6.7</v>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>56.21533333333333</v>
+        <v>56215.33333333334</v>
       </c>
       <c r="D71" t="n">
         <v>4.9</v>
@@ -3013,7 +3013,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>116.942</v>
+        <v>116942</v>
       </c>
       <c r="D72" t="n">
         <v>1.8</v>
@@ -3049,7 +3049,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1415.762666666667</v>
+        <v>1415762.666666667</v>
       </c>
       <c r="D73" t="n">
         <v>2.9</v>
@@ -3085,7 +3085,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>833.9530000000001</v>
+        <v>833953</v>
       </c>
       <c r="D74" t="n">
         <v>3.4</v>
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>935.8233333333333</v>
+        <v>935823.3333333334</v>
       </c>
       <c r="D75" t="n">
         <v>4.9</v>
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1252.520333333333</v>
+        <v>1252520.333333333</v>
       </c>
       <c r="D76" t="n">
         <v>14.4</v>
@@ -3193,7 +3193,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>823.7020000000001</v>
+        <v>823702</v>
       </c>
       <c r="D77" t="n">
         <v>10.7</v>
@@ -3229,7 +3229,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>438.1393333333333</v>
+        <v>438139.3333333333</v>
       </c>
       <c r="D78" t="n">
         <v>4.6</v>
@@ -3265,7 +3265,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1794.578666666667</v>
+        <v>1794578.666666667</v>
       </c>
       <c r="D79" t="n">
         <v>2.7</v>
@@ -3301,7 +3301,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>63.13399999999999</v>
+        <v>63134</v>
       </c>
       <c r="D80" t="n">
         <v>7.6</v>
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>49.36833333333333</v>
+        <v>49368.33333333334</v>
       </c>
       <c r="D81" t="n">
         <v>1.445454545454546</v>
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4134.183</v>
+        <v>4134183</v>
       </c>
       <c r="D82" t="n">
         <v>4.3</v>
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>775.5136666666667</v>
+        <v>775513.6666666666</v>
       </c>
       <c r="D83" t="n">
         <v>2.5</v>
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>177.3906666666667</v>
+        <v>177390.6666666667</v>
       </c>
       <c r="D84" t="n">
         <v>2.8</v>
@@ -3481,7 +3481,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>301.2693333333333</v>
+        <v>301269.3333333333</v>
       </c>
       <c r="D85" t="n">
         <v>5.1</v>
@@ -3517,7 +3517,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>429.4949999999999</v>
+        <v>429495</v>
       </c>
       <c r="D86" t="n">
         <v>4.3</v>
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>285.2923333333333</v>
+        <v>285292.3333333333</v>
       </c>
       <c r="D87" t="n">
         <v>11.2</v>
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>103.0066666666667</v>
+        <v>103006.6666666667</v>
       </c>
       <c r="D88" t="n">
         <v>2.3</v>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1742.14</v>
+        <v>1742140</v>
       </c>
       <c r="D89" t="n">
         <v>3.5</v>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1515.247666666667</v>
+        <v>1515247.666666667</v>
       </c>
       <c r="D90" t="n">
         <v>10.4</v>
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>601.3126666666667</v>
+        <v>601312.6666666666</v>
       </c>
       <c r="D91" t="n">
         <v>1.6</v>
@@ -3733,7 +3733,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>382.1156666666666</v>
+        <v>382115.6666666667</v>
       </c>
       <c r="D92" t="n">
         <v>4.461538461538462</v>
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>4437.454</v>
+        <v>4437454</v>
       </c>
       <c r="D93" t="n">
         <v>4.53</v>
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>76.33733333333333</v>
+        <v>76337.33333333333</v>
       </c>
       <c r="D94" t="n">
         <v>17.7</v>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>7854.294666666666</v>
+        <v>7854294.666666667</v>
       </c>
       <c r="D95" t="n">
         <v>3.7</v>
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3706.876333333334</v>
+        <v>3706876.333333333</v>
       </c>
       <c r="D96" t="n">
         <v>3.9</v>
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2119.721</v>
+        <v>2119721</v>
       </c>
       <c r="D97" t="n">
         <v>3</v>
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>21192.942</v>
+        <v>21192942</v>
       </c>
       <c r="D98" t="n">
         <v>23.1</v>
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2274.471</v>
+        <v>2274471</v>
       </c>
       <c r="D99" t="n">
         <v>22.5</v>
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>5097.207333333333</v>
+        <v>5097207.333333333</v>
       </c>
       <c r="D100" t="n">
         <v>33</v>
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>4196.186333333334</v>
+        <v>4196186.333333333</v>
       </c>
       <c r="D101" t="n">
         <v>40.7</v>
@@ -4093,7 +4093,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>14899.11633333333</v>
+        <v>14899116.33333333</v>
       </c>
       <c r="D102" t="n">
         <v>15.9</v>
@@ -4129,7 +4129,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1090.037</v>
+        <v>1090037</v>
       </c>
       <c r="D103" t="n">
         <v>17.1</v>
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2068.218333333334</v>
+        <v>2068218.333333333</v>
       </c>
       <c r="D104" t="n">
         <v>6.7</v>
@@ -4201,7 +4201,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>104.622</v>
+        <v>104622</v>
       </c>
       <c r="D105" t="n">
         <v>31.9</v>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>11003.37966666667</v>
+        <v>11003379.66666667</v>
       </c>
       <c r="D106" t="n">
         <v>21.7</v>
@@ -4273,7 +4273,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>32.21933333333333</v>
+        <v>32219.33333333333</v>
       </c>
       <c r="D107" t="n">
         <v>8.699999999999999</v>
@@ -4309,7 +4309,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1140.835333333333</v>
+        <v>1140835.333333333</v>
       </c>
       <c r="D108" t="n">
         <v>9.300000000000001</v>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>76443.10400000001</v>
+        <v>76443104</v>
       </c>
       <c r="D109" t="n">
         <v>31.5</v>
@@ -4381,7 +4381,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>20.428</v>
+        <v>20428</v>
       </c>
       <c r="D110" t="n">
         <v>14.8</v>
@@ -4417,7 +4417,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2954.6</v>
+        <v>2954600</v>
       </c>
       <c r="D111" t="n">
         <v>19.5</v>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1861.383333333333</v>
+        <v>1861383.333333333</v>
       </c>
       <c r="D112" t="n">
         <v>18.3</v>
@@ -4489,7 +4489,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1210.857666666667</v>
+        <v>1210857.666666667</v>
       </c>
       <c r="D113" t="n">
         <v>16.3</v>
@@ -4525,7 +4525,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>38694.96933333333</v>
+        <v>38694969.33333334</v>
       </c>
       <c r="D114" t="n">
         <v>2.4</v>
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>0.6573333333333333</v>
+        <v>657.3333333333334</v>
       </c>
       <c r="D115" t="n">
         <v>14.48334201388889</v>
@@ -4597,7 +4597,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>55.10400000000001</v>
+        <v>55104</v>
       </c>
       <c r="D116" t="n">
         <v>4.6</v>
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>10.854</v>
+        <v>10854</v>
       </c>
       <c r="D117" t="n">
         <v>6.9</v>
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>530.462</v>
+        <v>530462</v>
       </c>
       <c r="D118" t="n">
         <v>24.3</v>
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1514.116666666667</v>
+        <v>1514116.666666667</v>
       </c>
       <c r="D119" t="n">
         <v>15.3</v>
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2.858333333333333</v>
+        <v>2858.333333333333</v>
       </c>
       <c r="D120" t="n">
         <v>11.9</v>
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>8.086666666666668</v>
+        <v>8086.666666666667</v>
       </c>
       <c r="D121" t="n">
         <v>14.48334201388889</v>
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>235.3286666666667</v>
+        <v>235328.6666666667</v>
       </c>
       <c r="D122" t="n">
         <v>1.9</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>0.9923333333333333</v>
+        <v>992.3333333333334</v>
       </c>
       <c r="D123" t="n">
         <v>3.8</v>
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>0.082</v>
+        <v>82</v>
       </c>
       <c r="D124" t="n">
         <v>14.48334201388889</v>
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>0.656</v>
+        <v>656</v>
       </c>
       <c r="D125" t="n">
         <v>17.684</v>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>819.1286666666666</v>
+        <v>819128.6666666666</v>
       </c>
       <c r="D126" t="n">
         <v>27.8</v>
@@ -4993,7 +4993,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>6401.461333333333</v>
+        <v>6401461.333333333</v>
       </c>
       <c r="D127" t="n">
         <v>16.7</v>
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>905.511</v>
+        <v>905511</v>
       </c>
       <c r="D128" t="n">
         <v>0.4</v>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>18.856</v>
+        <v>18856</v>
       </c>
       <c r="D129" t="n">
         <v>3.4</v>
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>69.12133333333334</v>
+        <v>69121.33333333333</v>
       </c>
       <c r="D130" t="n">
         <v>16.2</v>
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>7.870333333333334</v>
+        <v>7870.333333333333</v>
       </c>
       <c r="D131" t="n">
         <v>0.8</v>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>0.7313333333333333</v>
+        <v>731.3333333333334</v>
       </c>
       <c r="D132" t="n">
         <v>2.9</v>
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>29.333</v>
+        <v>29333</v>
       </c>
       <c r="D133" t="n">
         <v>11.7</v>
@@ -5245,7 +5245,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>4785.569666666666</v>
+        <v>4785569.666666667</v>
       </c>
       <c r="D134" t="n">
         <v>9.699999999999999</v>

</xml_diff>